<commit_message>
HW: Cost estimation updated
</commit_message>
<xml_diff>
--- a/hw/Cost Estimation.xlsx
+++ b/hw/Cost Estimation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Daten\Daniel\ele\bat_source\hw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F41806E1-C7D2-4C35-9B59-1B78902EDBFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC58493-97D2-4BCB-95D4-0F3A2F975057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17325" tabRatio="735" firstSheet="1" activeTab="4" xr2:uid="{23E9BD06-C4F9-4485-BC66-1FB5ADDDACFE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17325" tabRatio="735" firstSheet="3" activeTab="7" xr2:uid="{23E9BD06-C4F9-4485-BC66-1FB5ADDDACFE}"/>
   </bookViews>
   <sheets>
     <sheet name="Bestellungen Prototypen" sheetId="3" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Kostenabschätzung" sheetId="6" r:id="rId5"/>
     <sheet name="Kostenabschätzung Serie Detail" sheetId="2" r:id="rId6"/>
     <sheet name="Kostenabschätzung Serie Det (2)" sheetId="7" r:id="rId7"/>
+    <sheet name="Kostenabschätzung Prototyp 2" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="408">
   <si>
     <t>LCD</t>
   </si>
@@ -1158,6 +1159,114 @@
   </si>
   <si>
     <t>Before FSG 25</t>
+  </si>
+  <si>
+    <t>Kostenabschätzung Prototyp 2</t>
+  </si>
+  <si>
+    <t>PS1-1BA</t>
+  </si>
+  <si>
+    <t>PS1-2BA</t>
+  </si>
+  <si>
+    <t>Stückpreis</t>
+  </si>
+  <si>
+    <t>Batterie</t>
+  </si>
+  <si>
+    <t>Typ</t>
+  </si>
+  <si>
+    <t>Hauptplatine</t>
+  </si>
+  <si>
+    <t>UI Platine</t>
+  </si>
+  <si>
+    <t>Anzahl pro Gerät</t>
+  </si>
+  <si>
+    <t>TYN30-600</t>
+  </si>
+  <si>
+    <t>GDT</t>
+  </si>
+  <si>
+    <t>Buchse rot</t>
+  </si>
+  <si>
+    <t>Buchse schwarz</t>
+  </si>
+  <si>
+    <t>Relais</t>
+  </si>
+  <si>
+    <t>Transformer</t>
+  </si>
+  <si>
+    <t>Taster</t>
+  </si>
+  <si>
+    <t>Temperatursensor</t>
+  </si>
+  <si>
+    <t>Stiftleiste 12x2</t>
+  </si>
+  <si>
+    <t>Buchsenleiste 12x2</t>
+  </si>
+  <si>
+    <t>Prototypen</t>
+  </si>
+  <si>
+    <t>Währung</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>EUR</t>
+  </si>
+  <si>
+    <t>CHF</t>
+  </si>
+  <si>
+    <t>Gesamtkosten</t>
+  </si>
+  <si>
+    <t>MCP6N11-001</t>
+  </si>
+  <si>
+    <t>Hauptplatine Bestückung</t>
+  </si>
+  <si>
+    <t>NHD-2.4-240320AF-CSXP-2MM Rev2B</t>
+  </si>
+  <si>
+    <t>UI Platine Bestückung</t>
+  </si>
+  <si>
+    <t>B88069X2180S102</t>
+  </si>
+  <si>
+    <t>803-87-024-10-001101</t>
+  </si>
+  <si>
+    <t>NRSE104F3380B1F</t>
+  </si>
+  <si>
+    <t>PRPC012DAAN-RC</t>
+  </si>
+  <si>
+    <t>304-03-423</t>
+  </si>
+  <si>
+    <t>303-95-366</t>
+  </si>
+  <si>
+    <t>Zubehör</t>
   </si>
 </sst>
 </file>
@@ -6148,11 +6257,11 @@
         <v>93.7</v>
       </c>
       <c r="G6">
-        <f t="shared" ref="G6:H35" si="1">C6/C$4</f>
+        <f t="shared" ref="G6:H14" si="1">C6/C$4</f>
         <v>3.7480000000000002</v>
       </c>
       <c r="I6">
-        <f t="shared" ref="I6:I35" si="2">E6/D$4</f>
+        <f t="shared" ref="I6:I14" si="2">E6/D$4</f>
         <v>3.7480000000000002</v>
       </c>
       <c r="K6" t="s">
@@ -7000,6 +7109,886 @@
       <c r="I37">
         <f t="shared" si="6"/>
         <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D850909C-D7B8-417A-8365-583D48149159}">
+  <dimension ref="A1:J29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.42578125" customWidth="1"/>
+    <col min="2" max="2" width="33.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>372</v>
+      </c>
+      <c r="F1" t="s">
+        <v>391</v>
+      </c>
+      <c r="G1">
+        <f>G2/F2</f>
+        <v>223.52000000000004</v>
+      </c>
+      <c r="I1" t="s">
+        <v>357</v>
+      </c>
+      <c r="J1">
+        <f>J2/I2</f>
+        <v>223.51999999999998</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <f>SUM(G4:G1048576)</f>
+        <v>1117.6000000000001</v>
+      </c>
+      <c r="I2">
+        <v>15</v>
+      </c>
+      <c r="J2">
+        <f>SUM(J4:J1048576)</f>
+        <v>3352.7999999999997</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>350</v>
+      </c>
+      <c r="B3" t="s">
+        <v>377</v>
+      </c>
+      <c r="C3" t="s">
+        <v>375</v>
+      </c>
+      <c r="D3" t="s">
+        <v>392</v>
+      </c>
+      <c r="E3" t="s">
+        <v>380</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" t="s">
+        <v>396</v>
+      </c>
+      <c r="I3" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>378</v>
+      </c>
+      <c r="B4" t="s">
+        <v>373</v>
+      </c>
+      <c r="C4">
+        <f>110.01/5</f>
+        <v>22.002000000000002</v>
+      </c>
+      <c r="D4" t="s">
+        <v>393</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <f>E4*F$2</f>
+        <v>5</v>
+      </c>
+      <c r="G4">
+        <f>F4*C4</f>
+        <v>110.01000000000002</v>
+      </c>
+      <c r="I4">
+        <f>E4*I$2</f>
+        <v>15</v>
+      </c>
+      <c r="J4">
+        <f>C4*I4</f>
+        <v>330.03000000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>398</v>
+      </c>
+      <c r="B5" t="s">
+        <v>373</v>
+      </c>
+      <c r="C5">
+        <f>461.62/5</f>
+        <v>92.323999999999998</v>
+      </c>
+      <c r="D5" t="s">
+        <v>393</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <f>E5*F$2</f>
+        <v>5</v>
+      </c>
+      <c r="G5">
+        <f>F5*C5</f>
+        <v>461.62</v>
+      </c>
+      <c r="I5">
+        <f>E5*I$2</f>
+        <v>15</v>
+      </c>
+      <c r="J5">
+        <f>C5*I5</f>
+        <v>1384.86</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>376</v>
+      </c>
+      <c r="B6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6">
+        <v>2.25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>394</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <f t="shared" ref="F6:F29" si="0">E6*F$2</f>
+        <v>20</v>
+      </c>
+      <c r="G6">
+        <f>F6*C6</f>
+        <v>45</v>
+      </c>
+      <c r="I6">
+        <f t="shared" ref="I6:I26" si="1">E6*I$2</f>
+        <v>60</v>
+      </c>
+      <c r="J6">
+        <f t="shared" ref="J6:J26" si="2">C6*I6</f>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" t="s">
+        <v>381</v>
+      </c>
+      <c r="C7">
+        <v>1.04</v>
+      </c>
+      <c r="D7" t="s">
+        <v>395</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G7">
+        <f>F7*C7</f>
+        <v>5.2</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="2"/>
+        <v>15.600000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8">
+        <v>3061334</v>
+      </c>
+      <c r="C8">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="D8" t="s">
+        <v>395</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="G8">
+        <f>F8*C8</f>
+        <v>44</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="2"/>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>110</v>
+      </c>
+      <c r="B9">
+        <v>3576</v>
+      </c>
+      <c r="C9">
+        <v>4</v>
+      </c>
+      <c r="D9" t="s">
+        <v>395</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G9">
+        <f>F9*C9</f>
+        <v>20</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="2"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>382</v>
+      </c>
+      <c r="B10" t="s">
+        <v>401</v>
+      </c>
+      <c r="C10">
+        <v>1.41</v>
+      </c>
+      <c r="D10" t="s">
+        <v>395</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G10">
+        <f>F10*C10</f>
+        <v>7.05</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="2"/>
+        <v>21.15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>383</v>
+      </c>
+      <c r="B11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11">
+        <v>3.9020000000000001</v>
+      </c>
+      <c r="D11" t="s">
+        <v>395</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="G11">
+        <f>F11*C11</f>
+        <v>39.020000000000003</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="2"/>
+        <v>117.06</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>384</v>
+      </c>
+      <c r="B12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12">
+        <v>4.4859999999999998</v>
+      </c>
+      <c r="D12" t="s">
+        <v>395</v>
+      </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="G12">
+        <f>F12*C12</f>
+        <v>44.86</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="2"/>
+        <v>134.57999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>390</v>
+      </c>
+      <c r="B13" t="s">
+        <v>402</v>
+      </c>
+      <c r="C13">
+        <v>2.54</v>
+      </c>
+      <c r="D13" t="s">
+        <v>395</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G13">
+        <f>F13*C13</f>
+        <v>12.7</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="2"/>
+        <v>38.1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>385</v>
+      </c>
+      <c r="B14" t="s">
+        <v>98</v>
+      </c>
+      <c r="C14">
+        <v>2.4300000000000002</v>
+      </c>
+      <c r="D14" t="s">
+        <v>395</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G14">
+        <f>F14*C14</f>
+        <v>12.15</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="2"/>
+        <v>36.450000000000003</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>386</v>
+      </c>
+      <c r="D15" t="s">
+        <v>395</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G15">
+        <f>F15*C15</f>
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>388</v>
+      </c>
+      <c r="B16" t="s">
+        <v>403</v>
+      </c>
+      <c r="C16">
+        <v>0.27</v>
+      </c>
+      <c r="D16" t="s">
+        <v>395</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G16">
+        <f>F16*C16</f>
+        <v>1.35</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="2"/>
+        <v>4.0500000000000007</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>387</v>
+      </c>
+      <c r="B17" t="s">
+        <v>109</v>
+      </c>
+      <c r="C17">
+        <v>0.23</v>
+      </c>
+      <c r="D17" t="s">
+        <v>395</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G17">
+        <f>F17*C17</f>
+        <v>1.1500000000000001</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="2"/>
+        <v>3.45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>135</v>
+      </c>
+      <c r="B18" t="s">
+        <v>397</v>
+      </c>
+      <c r="C18">
+        <v>1.38</v>
+      </c>
+      <c r="D18" t="s">
+        <v>395</v>
+      </c>
+      <c r="E18">
+        <v>3</v>
+      </c>
+      <c r="F18">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="G18">
+        <f>F18*C18</f>
+        <v>20.7</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="2"/>
+        <v>62.099999999999994</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F19">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <f>F19*C19</f>
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>379</v>
+      </c>
+      <c r="B20" t="s">
+        <v>374</v>
+      </c>
+      <c r="C20">
+        <f>10.94/5</f>
+        <v>2.1879999999999997</v>
+      </c>
+      <c r="D20" t="s">
+        <v>393</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G20">
+        <f>F20*C20</f>
+        <v>10.939999999999998</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="2"/>
+        <v>32.819999999999993</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>400</v>
+      </c>
+      <c r="B21" t="s">
+        <v>374</v>
+      </c>
+      <c r="C21">
+        <f>94.01/5</f>
+        <v>18.802</v>
+      </c>
+      <c r="D21" t="s">
+        <v>393</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G21">
+        <f>F21*C21</f>
+        <v>94.009999999999991</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="2"/>
+        <v>282.02999999999997</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>389</v>
+      </c>
+      <c r="B22" t="s">
+        <v>404</v>
+      </c>
+      <c r="C22">
+        <v>0.52</v>
+      </c>
+      <c r="D22" t="s">
+        <v>395</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G22">
+        <f>F22*C22</f>
+        <v>2.6</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="2"/>
+        <v>7.8000000000000007</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" t="s">
+        <v>399</v>
+      </c>
+      <c r="C23">
+        <v>15</v>
+      </c>
+      <c r="D23" t="s">
+        <v>393</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G23">
+        <f>F23*C23</f>
+        <v>75</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="2"/>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B24" t="s">
+        <v>81</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24" t="s">
+        <v>395</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G24">
+        <f>F24*C24</f>
+        <v>5</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J24">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" t="s">
+        <v>405</v>
+      </c>
+      <c r="C25">
+        <v>5.2430000000000003</v>
+      </c>
+      <c r="D25" t="s">
+        <v>395</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G25">
+        <f>F25*C25</f>
+        <v>26.215000000000003</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J25">
+        <f t="shared" si="2"/>
+        <v>78.64500000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>72</v>
+      </c>
+      <c r="B26" t="s">
+        <v>406</v>
+      </c>
+      <c r="C26">
+        <v>5.8049999999999997</v>
+      </c>
+      <c r="D26" t="s">
+        <v>395</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G26">
+        <f>F26*C26</f>
+        <v>29.024999999999999</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="2"/>
+        <v>87.074999999999989</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>51</v>
+      </c>
+      <c r="C28">
+        <v>5</v>
+      </c>
+      <c r="D28" t="s">
+        <v>394</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G28">
+        <f>F28*C28</f>
+        <v>25</v>
+      </c>
+      <c r="I28">
+        <f t="shared" ref="I28:I29" si="3">E28*I$2</f>
+        <v>15</v>
+      </c>
+      <c r="J28">
+        <f t="shared" ref="J28:J29" si="4">C28*I28</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>407</v>
+      </c>
+      <c r="C29">
+        <v>5</v>
+      </c>
+      <c r="D29" t="s">
+        <v>394</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G29">
+        <f>F29*C29</f>
+        <v>25</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="3"/>
+        <v>15</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="4"/>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
HW: Cost estimation updated with transformer
</commit_message>
<xml_diff>
--- a/hw/Cost Estimation.xlsx
+++ b/hw/Cost Estimation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Daten\Daniel\ele\bat_source\hw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC58493-97D2-4BCB-95D4-0F3A2F975057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{266E058E-8168-4BE8-84B2-8276D463D492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17325" tabRatio="735" firstSheet="3" activeTab="7" xr2:uid="{23E9BD06-C4F9-4485-BC66-1FB5ADDDACFE}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="423">
   <si>
     <t>LCD</t>
   </si>
@@ -1267,6 +1267,51 @@
   </si>
   <si>
     <t>Zubehör</t>
+  </si>
+  <si>
+    <t>Trafoplatine</t>
+  </si>
+  <si>
+    <t>PS1-100AA</t>
+  </si>
+  <si>
+    <t>Diode</t>
+  </si>
+  <si>
+    <t>Keramikkondensator</t>
+  </si>
+  <si>
+    <t>Widerstand 10M/0603 HV</t>
+  </si>
+  <si>
+    <t>RV0603FR-0710ML</t>
+  </si>
+  <si>
+    <t>Wickelkörper</t>
+  </si>
+  <si>
+    <t>US1NWF-7</t>
+  </si>
+  <si>
+    <t>CHV1210N1K5333KXT</t>
+  </si>
+  <si>
+    <t>B65822F1008T002X</t>
+  </si>
+  <si>
+    <t>B65805C0100A033</t>
+  </si>
+  <si>
+    <t>Ferritkern (Set)</t>
+  </si>
+  <si>
+    <t>Klammer für Kern</t>
+  </si>
+  <si>
+    <t>B65806J2204X000</t>
+  </si>
+  <si>
+    <t>Draht 0.106mm Grad 2</t>
   </si>
 </sst>
 </file>
@@ -7118,14 +7163,14 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D850909C-D7B8-417A-8365-583D48149159}">
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" customWidth="1"/>
     <col min="2" max="2" width="33.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>372</v>
       </c>
@@ -7134,33 +7179,49 @@
       </c>
       <c r="G1">
         <f>G2/F2</f>
-        <v>223.52000000000004</v>
+        <v>230.93520000000004</v>
+      </c>
+      <c r="H1">
+        <f>G1*1.088</f>
+        <v>251.25749760000005</v>
       </c>
       <c r="I1" t="s">
         <v>357</v>
       </c>
       <c r="J1">
         <f>J2/I2</f>
-        <v>223.51999999999998</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+        <v>230.93519999999998</v>
+      </c>
+      <c r="K1">
+        <f>J1*1.088</f>
+        <v>251.25749759999999</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F2">
         <v>5</v>
       </c>
       <c r="G2">
         <f>SUM(G4:G1048576)</f>
-        <v>1117.6000000000001</v>
+        <v>1154.6760000000002</v>
+      </c>
+      <c r="H2">
+        <f>G2*1.088</f>
+        <v>1256.2874880000002</v>
       </c>
       <c r="I2">
         <v>15</v>
       </c>
       <c r="J2">
         <f>SUM(J4:J1048576)</f>
-        <v>3352.7999999999997</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+        <v>3464.0279999999998</v>
+      </c>
+      <c r="K2">
+        <f>J2*1.088</f>
+        <v>3768.8624639999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>350</v>
       </c>
@@ -7189,7 +7250,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>378</v>
       </c>
@@ -7211,7 +7272,7 @@
         <v>5</v>
       </c>
       <c r="G4">
-        <f>F4*C4</f>
+        <f t="shared" ref="G4:G26" si="0">F4*C4</f>
         <v>110.01000000000002</v>
       </c>
       <c r="I4">
@@ -7223,7 +7284,7 @@
         <v>330.03000000000003</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>398</v>
       </c>
@@ -7245,7 +7306,7 @@
         <v>5</v>
       </c>
       <c r="G5">
-        <f>F5*C5</f>
+        <f t="shared" si="0"/>
         <v>461.62</v>
       </c>
       <c r="I5">
@@ -7257,7 +7318,7 @@
         <v>1384.86</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>376</v>
       </c>
@@ -7274,23 +7335,23 @@
         <v>4</v>
       </c>
       <c r="F6">
-        <f t="shared" ref="F6:F29" si="0">E6*F$2</f>
+        <f t="shared" ref="F6:F39" si="1">E6*F$2</f>
         <v>20</v>
       </c>
       <c r="G6">
-        <f>F6*C6</f>
+        <f t="shared" si="0"/>
         <v>45</v>
       </c>
       <c r="I6">
-        <f t="shared" ref="I6:I26" si="1">E6*I$2</f>
+        <f t="shared" ref="I6:I36" si="2">E6*I$2</f>
         <v>60</v>
       </c>
       <c r="J6">
-        <f t="shared" ref="J6:J26" si="2">C6*I6</f>
+        <f t="shared" ref="J6:J26" si="3">C6*I6</f>
         <v>135</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>105</v>
       </c>
@@ -7307,23 +7368,23 @@
         <v>1</v>
       </c>
       <c r="F7">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G7">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G7">
-        <f>F7*C7</f>
         <v>5.2</v>
       </c>
       <c r="I7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>15.600000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>113</v>
       </c>
@@ -7340,23 +7401,23 @@
         <v>2</v>
       </c>
       <c r="F8">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="G8">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="G8">
-        <f>F8*C8</f>
         <v>44</v>
       </c>
       <c r="I8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="J8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>132</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>110</v>
       </c>
@@ -7373,23 +7434,23 @@
         <v>1</v>
       </c>
       <c r="F9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G9">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G9">
-        <f>F9*C9</f>
         <v>20</v>
       </c>
       <c r="I9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>382</v>
       </c>
@@ -7406,23 +7467,23 @@
         <v>1</v>
       </c>
       <c r="F10">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G10">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G10">
-        <f>F10*C10</f>
         <v>7.05</v>
       </c>
       <c r="I10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>21.15</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>383</v>
       </c>
@@ -7439,23 +7500,23 @@
         <v>2</v>
       </c>
       <c r="F11">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="G11">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="G11">
-        <f>F11*C11</f>
         <v>39.020000000000003</v>
       </c>
       <c r="I11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="J11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>117.06</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>384</v>
       </c>
@@ -7472,23 +7533,23 @@
         <v>2</v>
       </c>
       <c r="F12">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="G12">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="G12">
-        <f>F12*C12</f>
         <v>44.86</v>
       </c>
       <c r="I12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="J12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>134.57999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>390</v>
       </c>
@@ -7505,23 +7566,23 @@
         <v>1</v>
       </c>
       <c r="F13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G13">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G13">
-        <f>F13*C13</f>
         <v>12.7</v>
       </c>
       <c r="I13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>38.1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>385</v>
       </c>
@@ -7538,23 +7599,23 @@
         <v>1</v>
       </c>
       <c r="F14">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G14">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G14">
-        <f>F14*C14</f>
         <v>12.15</v>
       </c>
       <c r="I14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>36.450000000000003</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>386</v>
       </c>
@@ -7565,23 +7626,23 @@
         <v>1</v>
       </c>
       <c r="F15">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G15">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G15">
-        <f>F15*C15</f>
         <v>0</v>
       </c>
       <c r="I15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J15">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>388</v>
       </c>
@@ -7598,19 +7659,19 @@
         <v>1</v>
       </c>
       <c r="F16">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G16">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G16">
-        <f>F16*C16</f>
         <v>1.35</v>
       </c>
       <c r="I16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.0500000000000007</v>
       </c>
     </row>
@@ -7631,19 +7692,19 @@
         <v>1</v>
       </c>
       <c r="F17">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G17">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G17">
-        <f>F17*C17</f>
         <v>1.1500000000000001</v>
       </c>
       <c r="I17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.45</v>
       </c>
     </row>
@@ -7664,37 +7725,37 @@
         <v>3</v>
       </c>
       <c r="F18">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="G18">
         <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="G18">
-        <f>F18*C18</f>
         <v>20.7</v>
       </c>
       <c r="I18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>45</v>
       </c>
       <c r="J18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>62.099999999999994</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G19">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G19">
-        <f>F19*C19</f>
-        <v>0</v>
-      </c>
       <c r="I19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J19">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -7716,19 +7777,19 @@
         <v>1</v>
       </c>
       <c r="F20">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G20">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G20">
-        <f>F20*C20</f>
         <v>10.939999999999998</v>
       </c>
       <c r="I20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>32.819999999999993</v>
       </c>
     </row>
@@ -7750,19 +7811,19 @@
         <v>1</v>
       </c>
       <c r="F21">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G21">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G21">
-        <f>F21*C21</f>
         <v>94.009999999999991</v>
       </c>
       <c r="I21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>282.02999999999997</v>
       </c>
     </row>
@@ -7783,19 +7844,19 @@
         <v>1</v>
       </c>
       <c r="F22">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G22">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G22">
-        <f>F22*C22</f>
         <v>2.6</v>
       </c>
       <c r="I22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>7.8000000000000007</v>
       </c>
     </row>
@@ -7816,19 +7877,19 @@
         <v>1</v>
       </c>
       <c r="F23">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G23">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G23">
-        <f>F23*C23</f>
         <v>75</v>
       </c>
       <c r="I23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>225</v>
       </c>
     </row>
@@ -7849,19 +7910,19 @@
         <v>1</v>
       </c>
       <c r="F24">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G24">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="G24">
-        <f>F24*C24</f>
-        <v>5</v>
-      </c>
       <c r="I24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J24">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>15</v>
       </c>
     </row>
@@ -7882,19 +7943,19 @@
         <v>1</v>
       </c>
       <c r="F25">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G25">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="G25">
-        <f>F25*C25</f>
         <v>26.215000000000003</v>
       </c>
       <c r="I25">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="J25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>78.64500000000001</v>
       </c>
     </row>
@@ -7915,79 +7976,391 @@
         <v>1</v>
       </c>
       <c r="F26">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G26">
         <f t="shared" si="0"/>
+        <v>29.024999999999999</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="3"/>
+        <v>87.074999999999989</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="G26">
-        <f>F26*C26</f>
-        <v>29.024999999999999</v>
-      </c>
-      <c r="I26">
+      <c r="G27">
+        <f t="shared" ref="G27:G36" si="4">F27*C27</f>
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <f t="shared" ref="I27:I36" si="5">E27*I$2</f>
+        <v>15</v>
+      </c>
+      <c r="J27">
+        <f t="shared" ref="J27:J36" si="6">C27*I27</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>408</v>
+      </c>
+      <c r="B28" t="s">
+        <v>409</v>
+      </c>
+      <c r="C28">
+        <v>0.44</v>
+      </c>
+      <c r="D28" t="s">
+        <v>395</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="4"/>
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="5"/>
+        <v>15</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="6"/>
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>410</v>
+      </c>
+      <c r="B29" t="s">
+        <v>415</v>
+      </c>
+      <c r="C29">
+        <v>0.253</v>
+      </c>
+      <c r="D29" t="s">
+        <v>395</v>
+      </c>
+      <c r="E29">
+        <v>3</v>
+      </c>
+      <c r="F29">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="J26">
-        <f t="shared" si="2"/>
-        <v>87.074999999999989</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="G29">
+        <f t="shared" si="4"/>
+        <v>3.7949999999999999</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="5"/>
+        <v>45</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="6"/>
+        <v>11.385</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>411</v>
+      </c>
+      <c r="B30" t="s">
+        <v>416</v>
+      </c>
+      <c r="C30">
+        <v>0.34599999999999997</v>
+      </c>
+      <c r="D30" t="s">
+        <v>395</v>
+      </c>
+      <c r="E30">
+        <v>3</v>
+      </c>
+      <c r="F30">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="4"/>
+        <v>5.1899999999999995</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="5"/>
+        <v>45</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="6"/>
+        <v>15.569999999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>412</v>
+      </c>
+      <c r="B31" t="s">
+        <v>413</v>
+      </c>
+      <c r="C31">
+        <v>0.1118</v>
+      </c>
+      <c r="D31" t="s">
+        <v>395</v>
+      </c>
+      <c r="E31">
+        <v>9</v>
+      </c>
+      <c r="F31">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="4"/>
+        <v>5.0309999999999997</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="5"/>
+        <v>135</v>
+      </c>
+      <c r="J31">
+        <f t="shared" si="6"/>
+        <v>15.093</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>414</v>
+      </c>
+      <c r="B32" t="s">
+        <v>417</v>
+      </c>
+      <c r="C32">
+        <v>1.17</v>
+      </c>
+      <c r="D32" t="s">
+        <v>395</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G32">
+        <f t="shared" si="4"/>
+        <v>5.85</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="5"/>
+        <v>15</v>
+      </c>
+      <c r="J32">
+        <f t="shared" si="6"/>
+        <v>17.549999999999997</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>419</v>
+      </c>
+      <c r="B33" t="s">
+        <v>418</v>
+      </c>
+      <c r="C33">
+        <v>2.74</v>
+      </c>
+      <c r="D33" t="s">
+        <v>395</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G33">
+        <f t="shared" si="4"/>
+        <v>13.700000000000001</v>
+      </c>
+      <c r="I33">
+        <f t="shared" si="5"/>
+        <v>15</v>
+      </c>
+      <c r="J33">
+        <f t="shared" si="6"/>
+        <v>41.1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>420</v>
+      </c>
+      <c r="B34" t="s">
+        <v>421</v>
+      </c>
+      <c r="C34">
+        <v>0.13100000000000001</v>
+      </c>
+      <c r="D34" t="s">
+        <v>395</v>
+      </c>
+      <c r="E34">
+        <v>2</v>
+      </c>
+      <c r="F34">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="G34">
+        <f t="shared" si="4"/>
+        <v>1.31</v>
+      </c>
+      <c r="I34">
+        <f t="shared" si="5"/>
+        <v>30</v>
+      </c>
+      <c r="J34">
+        <f t="shared" si="6"/>
+        <v>3.93</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>361</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35" t="s">
+        <v>395</v>
+      </c>
+      <c r="E35">
+        <v>0.4</v>
+      </c>
+      <c r="F35">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="G35">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="I35">
+        <f t="shared" si="5"/>
+        <v>6</v>
+      </c>
+      <c r="J35">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>422</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="D36" t="s">
+        <v>395</v>
+      </c>
+      <c r="E36">
+        <v>6</v>
+      </c>
+      <c r="F36">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="G36">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <f t="shared" si="5"/>
+        <v>90</v>
+      </c>
+      <c r="J36">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>51</v>
       </c>
-      <c r="C28">
+      <c r="C38">
         <v>5</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D38" t="s">
         <v>394</v>
       </c>
-      <c r="E28">
-        <v>1</v>
-      </c>
-      <c r="F28">
-        <f t="shared" si="0"/>
+      <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="F38">
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="G28">
-        <f>F28*C28</f>
+      <c r="G38">
+        <f>F38*C38</f>
         <v>25</v>
       </c>
-      <c r="I28">
-        <f t="shared" ref="I28:I29" si="3">E28*I$2</f>
+      <c r="I38">
+        <f t="shared" ref="I38:I39" si="7">E38*I$2</f>
         <v>15</v>
       </c>
-      <c r="J28">
-        <f t="shared" ref="J28:J29" si="4">C28*I28</f>
+      <c r="J38">
+        <f t="shared" ref="J38:J39" si="8">C38*I38</f>
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>407</v>
       </c>
-      <c r="C29">
+      <c r="C39">
         <v>5</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D39" t="s">
         <v>394</v>
       </c>
-      <c r="E29">
-        <v>1</v>
-      </c>
-      <c r="F29">
-        <f t="shared" si="0"/>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="G29">
-        <f>F29*C29</f>
+      <c r="G39">
+        <f>F39*C39</f>
         <v>25</v>
       </c>
-      <c r="I29">
-        <f t="shared" si="3"/>
+      <c r="I39">
+        <f t="shared" si="7"/>
         <v>15</v>
       </c>
-      <c r="J29">
-        <f t="shared" si="4"/>
+      <c r="J39">
+        <f t="shared" si="8"/>
         <v>75</v>
       </c>
     </row>

</xml_diff>